<commit_message>
feat: complete SF02 lifecycle polish, quality gates, and security hardening
Close implement/converge gaps for interrupt, concurrency, persistence, and
connectivity; harden gitleaks, image-scan, service images, and dependency
locks; record T068 evidence while keeping public make dev fail-closed until
platform harness and activation complete.
</commit_message>
<xml_diff>
--- a/项目开发/V0.1_功能跟踪表.xlsx
+++ b/项目开发/V0.1_功能跟踪表.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="65">
   <si>
     <t>功能简介</t>
   </si>
@@ -34,15 +34,27 @@
     <t>2026-07-12</t>
   </si>
   <si>
+    <t>完成</t>
+  </si>
+  <si>
+    <t>0711</t>
+  </si>
+  <si>
+    <t>F02 用户账户服务（注册/登录）</t>
+  </si>
+  <si>
+    <t>开发中 ing</t>
+  </si>
+  <si>
+    <t>0722</t>
+  </si>
+  <si>
+    <t>F03 API Key 管理服务（接入/验证）</t>
+  </si>
+  <si>
     <t>调研</t>
   </si>
   <si>
-    <t>F02 用户账户服务（注册/登录）</t>
-  </si>
-  <si>
-    <t>F03 API Key 管理服务（接入/验证）</t>
-  </si>
-  <si>
     <t>F04 请求代理网关（OpenAI-compatible）</t>
   </si>
   <si>
@@ -194,9 +206,6 @@
   </si>
   <si>
     <t>正在编码实现中</t>
-  </si>
-  <si>
-    <t>完成</t>
   </si>
   <si>
     <t>已通过验收标准</t>
@@ -681,113 +690,117 @@
       <c r="C2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="2"/>
+      <c r="D2" s="2" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" s="2"/>
+        <v>9</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D4" s="2"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D5" s="2"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D6" s="2"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D7" s="2"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D8" s="2"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D9" s="2"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D10" s="2"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D11" s="2"/>
     </row>
@@ -823,25 +836,25 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D2" s="2"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D3" s="2"/>
     </row>
@@ -877,241 +890,241 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D2" s="2"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D3" s="2"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D4" s="2"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D5" s="2"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D6" s="2"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D7" s="2"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>26</v>
-      </c>
       <c r="C8" s="2" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D8" s="2"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D9" s="2"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D10" s="2"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D11" s="2"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D12" s="2"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D13" s="2"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D14" s="2"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D15" s="2"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D16" s="2"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D17" s="2"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D18" s="2"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D19" s="2"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D20" s="2"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="D21" s="2"/>
     </row>
@@ -1131,15 +1144,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>5</v>
@@ -1147,39 +1160,39 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B7" s="2">
         <v>10</v>
@@ -1191,32 +1204,32 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B9" s="2"/>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>60</v>
+        <v>6</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>